<commit_message>
Actualizando archivos de Scopus, WOS y scripts base
</commit_message>
<xml_diff>
--- a/RESULTS/report.xlsx
+++ b/RESULTS/report.xlsx
@@ -1,24 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stats_summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dedup_distribution" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw_counts_by_year" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw_citations_by_year" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="doc_types_by_year" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="stats_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PRISMA_Flow" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Methodology" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="quality_summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="dedup_distribution" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="raw_counts_by_year" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="raw_citations_by_year" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="doc_types_by_year" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'stats_summary'!$A$1:$B$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'dedup_distribution'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'raw_counts_by_year'!$A$1:$D$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'raw_citations_by_year'!$A$1:$D$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'doc_types_by_year'!$A$1:$P$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'stats_summary'!$A$1:$B$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PRISMA_Flow'!$A$1:$B$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Methodology'!$A$1:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'quality_summary'!$A$1:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'dedup_distribution'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'raw_counts_by_year'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'raw_citations_by_year'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'doc_types_by_year'!$A$1:$I$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,10 +447,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -463,190 +469,1036 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Loaded papers</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>8564</v>
-      </c>
+          <t>1. RAW DATA</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Omitted papers by document type</t>
+          <t>Loaded papers (Total)</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Total after omission</t>
+          <t>Loaded WoS</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8564</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Loaded WoS</t>
+          <t>Loaded WoS (%)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2952</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Loaded WoS (%)</t>
+          <t>Loaded Scopus</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>34.5</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Loaded Scopus</t>
+          <t>Loaded Scopus (%)</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>5612</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Loaded Scopus (%)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>65.5</v>
-      </c>
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Duplicated papers found</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>2403</v>
-      </c>
+          <t>2. DEDUPLICATION &amp; FILTERING TOTALS</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Duplicated papers found (%)</t>
+          <t>Internal Duplicates Removed (Scopus)</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>28.1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Removed duplicated WoS</t>
+          <t>Internal Duplicates Removed (WoS)</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>2412</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Removed duplicated WoS (%)</t>
+          <t>Quality Failed Records Removed (Scopus)</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>81.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Removed duplicated Scopus</t>
+          <t>Quality Failed Records Removed (WoS)</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Removed duplicated Scopus (%)</t>
+          <t>Cross-Database Duplicates Removed</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.4</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Total after duplicates removal</t>
+          <t>Post-Merge/Year Filtering Removed</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>5875</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Final WoS</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>540</v>
-      </c>
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Final WoS (%)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>9.199999999999999</v>
-      </c>
+          <t>3. FINAL DATASET</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Final Scopus</t>
+          <t>Total Removed (Scopus)</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5588</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Total Removed (Scopus %)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Total Removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Total Removed (WoS %)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Total Resulting Papers</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Final WoS</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Final WoS (%)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Final Scopus</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t>Final Scopus (%)</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B26" s="3" t="n">
+        <v>90.40000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>QUALITY CHECK (Before Filters)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Total records before quality filters</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Records with DOI</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Records with DOI (%)</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
         <v>95.09999999999999</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Records with Title</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Records with Title (%)</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Records with Authors</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Records with Authors (%)</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Records with Abstract</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Records with Abstract (%)</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>QUALITY CHECK (Final Dataset)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Total records after quality filters</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Records with DOI</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Records with DOI (%)</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>94.2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Records with Title</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Records with Title (%)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Records with Authors</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Records with Authors (%)</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Records with Abstract</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Records with Abstract (%)</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>PRISMA Step</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1. Records identified from Scopus</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1. Records identified from WoS</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Records identified (Total)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2. Internal duplicates removed (Scopus)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2. Internal duplicates removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Records after internal deduplication</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>3. Missing/Invalid DOIs removed (Scopus)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>3. Missing Titles removed (Scopus)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>3. Missing Authors removed (Scopus)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>3. Missing Abstracts removed (Scopus)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>4. Missing/Invalid DOIs removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>4. Missing Titles removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>4. Missing Authors removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>4. Missing Abstracts removed (WoS)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Records screened for quality</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>5. Cross-database duplicates removed</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>5. Post-Merge / Year filtering removed</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Total records included for synthesis</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Python/Library Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1. Data Loading</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Load CSVs from Scopus and Excel from WoS.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>pandas.read_csv, pandas.read_excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2. Internal Deduplication</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Remove duplicate rows within the same database based on Title.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>pandas.drop_duplicates(subset=['processed_title'])</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>3. Quality: DOI Cleaning</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Extract valid DOIs using regular expressions and remove empty.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>re.search(r'(10\.\d{4,9}/[-._;()/:a-z0-9]+)'), df[df['DOI'] != '']</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>4. Quality: Missing Titles</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Remove records where the title is completely empty.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>df[df['Title'].fillna('').str.strip() != '']</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>5. Quality: Missing Authors</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Remove records where authors are missing.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>df[df['Authors'].fillna('').str.strip() != '']</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>6. Quality: Missing Abstracts</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Remove records where abstract is missing.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>df[df['Abstract'].fillna('').str.strip() != '']</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>7. Cross-Deduplication</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Fuzzy matching to find overlapping titles between Scopus and WoS.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>thefuzz.fuzz.token_set_ratio &gt; config.FUZZY_THRESHOLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>8. Merging</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Normalize WoS columns to Scopus schema and concatenate.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>pandas.concat([scopus, wos_normalized])</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>9. Enriching</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Add SCImago Quartiles and Metrics based on ISSN/Journal Title.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>pandas.merge(combined_df, scimago_df)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Total Records (Final)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DOIs - Valid</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>DOIs - Blank</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>DOIs - Valid (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>94.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Years - Valid</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Years - Missing</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Years - Valid (%)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Titles - Valid</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Titles - Blank</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Titles - Valid (%)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Keywords - With Data</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Keywords - Blank</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Keywords - With Data (%)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -702,19 +1554,19 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>540</v>
+        <v>15</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2412</v>
+        <v>115</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2952</v>
+        <v>130</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>18.3</v>
+        <v>11.5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>81.7</v>
+        <v>88.5</v>
       </c>
     </row>
     <row r="3">
@@ -724,19 +1576,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>5588</v>
+        <v>141</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>5612</v>
+        <v>179</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>99.59999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.4</v>
+        <v>21.2</v>
       </c>
     </row>
   </sheetData>
@@ -745,13 +1597,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -784,171 +1636,241 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>2015</v>
+        <v>2007</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>159</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>232</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>2016</v>
+        <v>2010</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>178</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>268</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>121</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>206</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>327</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2018</v>
+        <v>2012</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>263</v>
+        <v>1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>396</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>122</v>
+        <v>2</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>275</v>
+        <v>2</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>397</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>392</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>627</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>326</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>572</v>
+        <v>2</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>898</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>378</v>
+        <v>1</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>632</v>
+        <v>2</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>1010</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>369</v>
+        <v>2</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>632</v>
+        <v>4</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1001</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>466</v>
+        <v>3</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>851</v>
+        <v>7</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1317</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>618</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>1175</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>1793</v>
+      <c r="B17" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -981,189 +1903,252 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>2015</v>
+        <v>2007</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>3702</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>6646</v>
+        <v>2</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10348</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>2016</v>
+        <v>2010</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4921</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7081</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>12002</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7710</v>
+        <v>72</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>6748</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>14458</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2018</v>
+        <v>2012</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>8518</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>7148</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>15666</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>7635</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>6826</v>
+        <v>78</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>14461</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>13233</v>
+        <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10846</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>24079</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>20220</v>
+        <v>109</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>12452</v>
+        <v>171</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>32672</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>23725</v>
+        <v>44</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>9052</v>
+        <v>120</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>32777</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>24718</v>
+        <v>104</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>5669</v>
+        <v>249</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>30387</v>
+        <v>353</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>31814</v>
+        <v>104</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3565</v>
+        <v>101</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>35379</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>382</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>635</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>520</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>613</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>368</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>689</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1095</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>42613</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>1013</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>43626</v>
+      <c r="B17" s="3" t="n">
+        <v>1310</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1374</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1179,70 +2164,35 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Book chapter</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Book Chapter</t>
+          <t>Conference Paper</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Book chapter</t>
+          <t>Conference paper</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Conference Paper</t>
+          <t>Early Access</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Conference paper</t>
+          <t>Erratum</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Conference review</t>
+          <t>Retracted</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Data paper</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Early Access</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Editorial</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Erratum</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Letter</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>Retracted</t>
-        </is>
-      </c>
-      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
@@ -1250,556 +2200,470 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>2015</v>
+        <v>2007</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>163</v>
+        <v>0</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>2016</v>
+        <v>2010</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>180</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="3" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>237</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2018</v>
+        <v>2012</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>263</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>297</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>414</v>
+        <v>1</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>598</v>
+        <v>3</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P8" s="3" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>663</v>
+        <v>1</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>652</v>
+        <v>3</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>809</v>
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>1080</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>64</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="3" t="n">
+      <c r="B17" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>5</v>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P12"/>
+  <autoFilter ref="A1:I17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>